<commit_message>
Improved performance of agent based on stakeholder feedback
</commit_message>
<xml_diff>
--- a/test_student_data.xlsx
+++ b/test_student_data.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectives" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,36 +468,41 @@
           <t>Assignment 5</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Assignment 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>James</t>
+          <t>Sam</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Stevens</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SO100000</t>
+          <t>SO3000</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>james.davis0@university.edu</t>
+          <t>s0@university.edu</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -506,44 +512,49 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Joe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Stevens</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SO100001</t>
+          <t>SO3001</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>john.garcia1@university.edu</t>
+          <t>s1@university.edu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CIS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -553,49 +564,54 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>F</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Larry</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Clippard</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SO100002</t>
+          <t>SO3002</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>linda.miller2@university.edu</t>
+          <t>s2@university.edu</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -615,39 +631,44 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Chitofu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SO100003</t>
+          <t>SO3003</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>robert.johnson3@university.edu</t>
+          <t>s3@university.edu</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -657,49 +678,54 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>B</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Samples</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SO100004</t>
+          <t>SO3004</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>michael.miller4@university.edu</t>
+          <t>s4@university.edu</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -709,20 +735,25 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -731,27 +762,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Nipesh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jones</t>
+          <t>Schwartz</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SO100005</t>
+          <t>SO3005</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>linda.jones5@university.edu</t>
+          <t>s5@university.edu</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -761,72 +792,82 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jones</t>
+          <t>Clippard</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SO100006</t>
+          <t>SO3006</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>robert.jones6@university.edu</t>
+          <t>s6@university.edu</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -835,50 +876,55 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>James</t>
+          <t>Larry</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Mitra</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SO100007</t>
+          <t>SO3007</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>james.johnson7@university.edu</t>
+          <t>s7@university.edu</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CIS</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>E</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -887,27 +933,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Ivy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Clippard</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SO100008</t>
+          <t>SO3008</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>jennifer.garcia8@university.edu</t>
+          <t>s8@university.edu</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -917,7 +963,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -927,54 +973,59 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Ivy</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Stevens</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SO100009</t>
+          <t>SO3009</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>michael.davis9@university.edu</t>
+          <t>s9@university.edu</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -984,44 +1035,49 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Reshmi</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Brucker</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SO100010</t>
+          <t>SO3010</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>mary.smith10@university.edu</t>
+          <t>s10@university.edu</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CIS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1031,54 +1087,59 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>James</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>DeRousse</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SO100011</t>
+          <t>SO3011</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>james.miller11@university.edu</t>
+          <t>s11@university.edu</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1089,147 +1150,162 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>C</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Anderson</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SO100012</t>
+          <t>SO3012</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>linda.brown12@university.edu</t>
+          <t>s12@university.edu</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Kyle</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Mitra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SO100013</t>
+          <t>SO3013</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>mary.davis13@university.edu</t>
+          <t>s13@university.edu</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Reshmi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Schwartz</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SO100014</t>
+          <t>SO3014</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>michael.brown14@university.edu</t>
+          <t>s14@university.edu</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1239,54 +1315,59 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Larry</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Pant</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SO100015</t>
+          <t>SO3015</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>linda.garcia15@university.edu</t>
+          <t>s15@university.edu</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1295,6 +1376,11 @@
         </is>
       </c>
       <c r="J17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1303,32 +1389,32 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Ivy</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Pant</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SO100016</t>
+          <t>SO3016</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>jennifer.davis16@university.edu</t>
+          <t>s16@university.edu</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1338,7 +1424,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1348,34 +1434,39 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Clippard</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SO100017</t>
+          <t>SO3017</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>mary.garcia17@university.edu</t>
+          <t>s17@university.edu</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1395,10 +1486,15 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1407,27 +1503,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Luyanda</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Brucker</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SO100018</t>
+          <t>SO3018</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>mary.johnson18@university.edu</t>
+          <t>s18@university.edu</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1442,44 +1538,49 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Schwartz</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SO100019</t>
+          <t>SO3019</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>linda.garcia19@university.edu</t>
+          <t>s19@university.edu</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1489,54 +1590,59 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Nipesh</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Williams</t>
+          <t>Mitra</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SO100020</t>
+          <t>SO3020</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>john.williams20@university.edu</t>
+          <t>s20@university.edu</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1551,10 +1657,15 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1563,32 +1674,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Patricia</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Brucker</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SO100021</t>
+          <t>SO3021</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>patricia.miller21@university.edu</t>
+          <t>s21@university.edu</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1598,15 +1709,20 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
       <c r="J23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1615,27 +1731,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Miller</t>
+          <t>Samples</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SO100022</t>
+          <t>SO3022</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>jennifer.miller22@university.edu</t>
+          <t>s22@university.edu</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CIS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1650,15 +1766,20 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -1667,42 +1788,42 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Patricia</t>
+          <t>Ivy</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Samples</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SO100023</t>
+          <t>SO3023</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>patricia.davis23@university.edu</t>
+          <t>s23@university.edu</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1712,39 +1833,44 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Robert</t>
+          <t>Marilla</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jones</t>
+          <t>Clippard</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SO100024</t>
+          <t>SO3024</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>robert.jones24@university.edu</t>
+          <t>s24@university.edu</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Cyber Security</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1754,15 +1880,20 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1771,84 +1902,89 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Patricia</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Stevens</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SO100025</t>
+          <t>SO3025</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>patricia.davis25@university.edu</t>
+          <t>s25@university.edu</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CIS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>F</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Marilla</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Mitra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SO100026</t>
+          <t>SO3026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>john.johnson26@university.edu</t>
+          <t>s26@university.edu</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1858,15 +1994,20 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -1875,27 +2016,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Kyle</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Davis</t>
+          <t>Schwartz</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SO100027</t>
+          <t>SO3027</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>linda.davis27@university.edu</t>
+          <t>s27@university.edu</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1905,20 +2046,25 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1927,104 +2073,213 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>James</t>
+          <t>Lilly</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Bartlet</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SO100028</t>
+          <t>SO3028</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>james.smith28@university.edu</t>
+          <t>s28@university.edu</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
           <t>A</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Linda</t>
+          <t>Nipesh</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Smith</t>
+          <t>Schwartz</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SO100029</t>
+          <t>SO3029</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>linda.smith29@university.edu</t>
+          <t>s29@university.edu</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Computer Science</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Objective ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Objective Description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Assignments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CO-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Understanding Cyberspace attacks.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Assignment 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CO-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Demonstrate cyber defense techniques.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Assignment 2, Assignment 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CO-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Evaluate connected systems.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Assignment 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CO-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tool development and scripting.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Assignment 5, Assignment 6</t>
         </is>
       </c>
     </row>

</xml_diff>